<commit_message>
docs: add virtual lidar partition variant
</commit_message>
<xml_diff>
--- a/Autoware_Partition_Data_Flow.xlsx
+++ b/Autoware_Partition_Data_Flow.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="745" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="799" uniqueCount="124">
   <si>
     <t xml:space="preserve">파티션별 컴포넌트 구성</t>
   </si>
@@ -97,10 +97,96 @@
     <t xml:space="preserve">Sensing</t>
   </si>
   <si>
-    <t xml:space="preserve">현재 시험에서는 미사용</t>
-  </si>
-  <si>
-    <t xml:space="preserve">실제 센서 드라이버와 센서 데이터 전처리</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">가상 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">LiDAR </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">전처리 사용</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">RViz </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">장애물 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Pointcloud</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">의 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">voxel downsample</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">과 차량 영역 제거를 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">CPU</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로 처리</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">Localization</t>
@@ -160,11 +246,19 @@
   <si>
     <r>
       <rPr>
+        <sz val="10"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">가상 </t>
+    </r>
+    <r>
+      <rPr>
         <sz val="9"/>
         <rFont val="Malgun Gothic"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">Dummy Perception </t>
+      <t xml:space="preserve">LiDAR CPU </t>
     </r>
     <r>
       <rPr>
@@ -172,17 +266,25 @@
         <rFont val="Malgun Gothic"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">사용</t>
-    </r>
-  </si>
-  <si>
+      <t xml:space="preserve">검출 사용</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">전처리 </t>
+    </r>
     <r>
       <rPr>
         <sz val="9"/>
         <rFont val="Malgun Gothic"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">RViz </t>
+      <t xml:space="preserve">Pointcloud</t>
     </r>
     <r>
       <rPr>
@@ -190,7 +292,7 @@
         <rFont val="Malgun Gothic"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">더미 객체를 검출</t>
+      <t xml:space="preserve">를 군집화하고 형상 추정</t>
     </r>
     <r>
       <rPr>
@@ -222,23 +324,7 @@
         <rFont val="Malgun Gothic"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">예측 객체와 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="Malgun Gothic"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Pointcloud</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Malgun Gothic"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">로 변환</t>
+      <t xml:space="preserve">예측 객체로 변환</t>
     </r>
   </si>
   <si>
@@ -579,6 +665,30 @@
     <t xml:space="preserve">/simulation/dummy_perception_publisher/object_info</t>
   </si>
   <si>
+    <t xml:space="preserve">autoware_pointcloud_preprocessor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/sensing/lidar/virtual/voxel_grid_downsample_filter_node</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/sensing/lidar/virtual/pointcloud_raw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/sensing/lidar/virtual/crop_box_filter_node</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/sensing/lidar/concatenated/pointcloud</t>
+  </si>
+  <si>
+    <t xml:space="preserve">autoware_euclidean_cluster</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/perception/object_recognition/detection/virtual_lidar_euclidean_cluster</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/perception/obstacle_segmentation/pointcloud</t>
+  </si>
+  <si>
     <t xml:space="preserve">autoware_shape_estimation</t>
   </si>
   <si>
@@ -640,9 +750,6 @@
   </si>
   <si>
     <t xml:space="preserve">/planning/scenario_planning/lane_driving/motion_planning/obstacle_cruise_planner</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/perception/obstacle_segmentation/pointcloud</t>
   </si>
   <si>
     <t xml:space="preserve">autoware_autonomous_emergency_braking</t>
@@ -1131,7 +1238,7 @@
       <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="3" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1156,10 +1263,10 @@
       <c r="B8" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="4" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1282,7 +1389,7 @@
     <tabColor rgb="FFA56600"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="13.78"/>
@@ -1374,7 +1481,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
@@ -1385,7 +1492,7 @@
         <v>5</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>44</v>
@@ -1411,25 +1518,25 @@
         <v>5</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>48</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>49</v>
       </c>
       <c r="H7" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="I7" s="3" t="s">
         <v>52</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1440,141 +1547,141 @@
         <v>5</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>5</v>
       </c>
       <c r="E8" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="G8" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="H8" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="G8" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="H8" s="3" t="s">
+      <c r="I8" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="I8" s="3" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E9" s="3" t="s">
+      <c r="G9" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="H9" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="G9" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="H9" s="3" t="s">
+      <c r="I9" s="3" t="s">
         <v>58</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>19</v>
+      <c r="B10" s="2" t="s">
+        <v>5</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E10" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="G10" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="H10" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="G10" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="H10" s="3" t="s">
+      <c r="I10" s="3" t="s">
         <v>61</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="5" t="s">
-        <v>19</v>
+      <c r="B11" s="2" t="s">
+        <v>5</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F11" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="H11" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="G11" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="H11" s="3" t="s">
+      <c r="I11" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="I11" s="3" t="s">
+    </row>
+    <row r="12" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E12" s="3" t="s">
         <v>62</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>57</v>
       </c>
       <c r="F12" s="3" t="s">
         <v>65</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>66</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1591,19 +1698,19 @@
         <v>20</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1620,19 +1727,19 @@
         <v>20</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1649,19 +1756,19 @@
         <v>20</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1678,367 +1785,367 @@
         <v>20</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B17" s="6" t="s">
-        <v>24</v>
+      <c r="B17" s="5" t="s">
+        <v>19</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>69</v>
+        <v>55</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B18" s="6" t="s">
-        <v>24</v>
+      <c r="B18" s="5" t="s">
+        <v>19</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="F18" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="I21" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="G18" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="I19" s="3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="H20" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="I20" s="3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="G21" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="H21" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="I21" s="3" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="22" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B22" s="5" t="s">
-        <v>19</v>
+      <c r="B22" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>60</v>
+        <v>79</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>76</v>
+        <v>51</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>61</v>
+        <v>80</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>78</v>
+        <v>55</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>5</v>
+      <c r="B23" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="C23" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C24" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D23" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="G23" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="H23" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="I23" s="3" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>17</v>
-      </c>
       <c r="D24" s="3" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>45</v>
+        <v>83</v>
       </c>
       <c r="H24" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="I24" s="3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E25" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="I24" s="3" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>79</v>
-      </c>
       <c r="F25" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G25" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="G25" s="3" t="s">
-        <v>45</v>
-      </c>
       <c r="H25" s="3" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
       <c r="I25" s="3" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>19</v>
+    <row r="26" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>5</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="I26" s="3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E27" s="3" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B27" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>60</v>
-      </c>
       <c r="F27" s="3" t="s">
-        <v>63</v>
+        <v>87</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>19</v>
+        <v>89</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>63</v>
+        <v>86</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2055,16 +2162,16 @@
         <v>20</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>91</v>
+        <v>68</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>92</v>
+        <v>69</v>
       </c>
       <c r="I29" s="3" t="s">
         <v>93</v>
@@ -2084,16 +2191,16 @@
         <v>20</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>91</v>
+        <v>68</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>92</v>
+        <v>69</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I30" s="3" t="s">
         <v>94</v>
@@ -2113,19 +2220,19 @@
         <v>20</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>67</v>
+        <v>95</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>68</v>
+        <v>96</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2142,51 +2249,51 @@
         <v>20</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>67</v>
+        <v>95</v>
       </c>
       <c r="F32" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="G32" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="G32" s="3" t="s">
-        <v>68</v>
-      </c>
       <c r="H32" s="3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="I32" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E33" s="3" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="33" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B33" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D33" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E33" s="3" t="s">
-        <v>96</v>
-      </c>
       <c r="F33" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="G33" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="G33" s="3" t="s">
-        <v>97</v>
-      </c>
       <c r="H33" s="3" t="s">
-        <v>100</v>
+        <v>74</v>
       </c>
       <c r="I33" s="3" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
         <v>19</v>
       </c>
@@ -2200,135 +2307,135 @@
         <v>20</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>99</v>
+        <v>73</v>
       </c>
       <c r="F34" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="G34" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="H34" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="I34" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="G34" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="H34" s="3" t="s">
+    </row>
+    <row r="35" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="F35" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="I34" s="3" t="s">
+      <c r="G35" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="H35" s="3" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="35" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B35" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D35" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E35" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="F35" s="3" t="s">
+      <c r="I35" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="G35" s="3" t="s">
+    </row>
+    <row r="36" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E36" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="H35" s="3" t="s">
+      <c r="F36" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="I35" s="3" t="s">
+      <c r="G36" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="H36" s="3" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="36" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B36" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D36" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="F36" s="3" t="s">
+      <c r="I36" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="G36" s="3" t="s">
+    </row>
+    <row r="37" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E37" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="H36" s="3" t="s">
+      <c r="F37" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="I36" s="3" t="s">
+      <c r="G37" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="H37" s="3" t="s">
         <v>110</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D37" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E37" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="F37" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="G37" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="H37" s="3" t="s">
-        <v>81</v>
       </c>
       <c r="I37" s="3" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B38" s="5" t="s">
-        <v>19</v>
+    <row r="38" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>80</v>
+        <v>109</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>60</v>
+        <v>112</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>81</v>
+        <v>110</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>61</v>
+        <v>113</v>
       </c>
       <c r="I38" s="3" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2339,87 +2446,174 @@
         <v>24</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>24</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>80</v>
+        <v>112</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>81</v>
+        <v>113</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="I39" s="3" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B40" s="5" t="s">
-        <v>19</v>
+      <c r="B40" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="C40" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D40" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D40" s="3" t="s">
-        <v>20</v>
-      </c>
       <c r="E40" s="3" t="s">
-        <v>80</v>
+        <v>115</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>81</v>
+        <v>116</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="I40" s="3" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B41" s="6" t="s">
-        <v>24</v>
+      <c r="B41" s="5" t="s">
+        <v>19</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>28</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>105</v>
+        <v>68</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="H41" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="I41" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="F42" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="G42" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="H42" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="I42" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="F43" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="I41" s="3" t="s">
-        <v>114</v>
+      <c r="G43" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="H43" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="I43" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="F44" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="G44" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="H44" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="I44" s="3" t="s">
+        <v>121</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I41"/>
+  <autoFilter ref="A4:I44"/>
   <mergeCells count="1">
     <mergeCell ref="A1:I2"/>
   </mergeCells>
@@ -2439,7 +2633,7 @@
     <tabColor rgb="FF76528F"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="13.78"/>
@@ -2451,7 +2645,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2531,7 +2725,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
@@ -2542,7 +2736,7 @@
         <v>5</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>44</v>
@@ -2568,25 +2762,25 @@
         <v>5</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>48</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>49</v>
       </c>
       <c r="H7" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="I7" s="3" t="s">
         <v>52</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2597,141 +2791,141 @@
         <v>5</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>5</v>
       </c>
       <c r="E8" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="G8" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="H8" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="G8" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="H8" s="3" t="s">
+      <c r="I8" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="I8" s="3" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E9" s="3" t="s">
+      <c r="G9" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="H9" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="G9" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="H9" s="3" t="s">
+      <c r="I9" s="3" t="s">
         <v>58</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>19</v>
+      <c r="B10" s="2" t="s">
+        <v>5</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E10" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="G10" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="H10" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="G10" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="H10" s="3" t="s">
+      <c r="I10" s="3" t="s">
         <v>61</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="5" t="s">
-        <v>19</v>
+      <c r="B11" s="2" t="s">
+        <v>5</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F11" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="H11" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="G11" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="H11" s="3" t="s">
+      <c r="I11" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="I11" s="3" t="s">
+    </row>
+    <row r="12" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E12" s="3" t="s">
         <v>62</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>57</v>
       </c>
       <c r="F12" s="3" t="s">
         <v>65</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>66</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2748,19 +2942,19 @@
         <v>20</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2777,19 +2971,19 @@
         <v>20</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2806,19 +3000,19 @@
         <v>20</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2835,139 +3029,226 @@
         <v>20</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B17" s="6" t="s">
-        <v>24</v>
+      <c r="B17" s="5" t="s">
+        <v>19</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>69</v>
+        <v>55</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B18" s="6" t="s">
-        <v>24</v>
+      <c r="B18" s="5" t="s">
+        <v>19</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="F18" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="I21" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="G18" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="I19" s="3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="H20" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="I20" s="3" t="s">
-        <v>62</v>
+    </row>
+    <row r="22" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="I22" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I20"/>
+  <autoFilter ref="A4:I23"/>
   <mergeCells count="1">
     <mergeCell ref="A1:I2"/>
   </mergeCells>
@@ -2999,7 +3280,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3064,19 +3345,19 @@
         <v>20</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3093,19 +3374,19 @@
         <v>20</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3122,19 +3403,19 @@
         <v>5</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3151,19 +3432,19 @@
         <v>28</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="G8" s="3" t="s">
         <v>45</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3180,19 +3461,19 @@
         <v>30</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="G9" s="3" t="s">
         <v>45</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3209,19 +3490,19 @@
         <v>20</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3238,19 +3519,19 @@
         <v>20</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3267,19 +3548,19 @@
         <v>20</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3296,19 +3577,19 @@
         <v>20</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3325,19 +3606,19 @@
         <v>20</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3354,19 +3635,19 @@
         <v>20</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3383,19 +3664,19 @@
         <v>20</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3412,19 +3693,19 @@
         <v>20</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3441,19 +3722,19 @@
         <v>20</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3470,19 +3751,19 @@
         <v>24</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3499,19 +3780,19 @@
         <v>24</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3528,19 +3809,19 @@
         <v>28</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3557,19 +3838,19 @@
         <v>20</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3586,19 +3867,19 @@
         <v>24</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3615,19 +3896,19 @@
         <v>20</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3644,19 +3925,19 @@
         <v>24</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>